<commit_message>
New run with 10% Reserve margin
</commit_message>
<xml_diff>
--- a/NECP Scenario/Results/Regional Results/CHIOS_Capacity.xlsx
+++ b/NECP Scenario/Results/Regional Results/CHIOS_Capacity.xlsx
@@ -533,25 +533,25 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>3.345287652185967E-08</v>
+        <v>4.925438172011717E-08</v>
       </c>
       <c r="C3">
-        <v>3.370298887774326E-08</v>
+        <v>4.959412309395111E-08</v>
       </c>
       <c r="D3">
-        <v>0.0263654230997974</v>
+        <v>0.0255933198275285</v>
       </c>
       <c r="E3">
-        <v>0.026831814591222</v>
+        <v>0.0260384865967236</v>
       </c>
       <c r="F3">
-        <v>0.0268317815384821</v>
+        <v>0.0260384379387488</v>
       </c>
       <c r="G3">
-        <v>0.0004707832238522</v>
+        <v>0.0015688087752985</v>
       </c>
       <c r="H3">
-        <v>0.0004709337035298</v>
+        <v>0.0018923922124158</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -793,25 +793,25 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>0.4000000000065827</v>
+        <v>0.4000000000072</v>
       </c>
       <c r="C13">
-        <v>0.4000000000086269</v>
+        <v>0.400000000010201</v>
       </c>
       <c r="D13">
-        <v>0.4000000000130073</v>
+        <v>0.4000000000158112</v>
       </c>
       <c r="E13">
-        <v>0.4000000000238337</v>
+        <v>0.4000000000290729</v>
       </c>
       <c r="F13">
-        <v>0.4000000000407969</v>
+        <v>0.4000000000501866</v>
       </c>
       <c r="G13">
-        <v>0.4000000000751622</v>
+        <v>0.4000000000939304</v>
       </c>
       <c r="H13">
-        <v>0.4000000004241097</v>
+        <v>0.4000000005056124</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -1163,19 +1163,19 @@
         <v>0</v>
       </c>
       <c r="D27">
-        <v>0.08343043441969571</v>
+        <v>0.08219256620403689</v>
       </c>
       <c r="E27">
-        <v>0.1345458987147521</v>
+        <v>0.1257985652780935</v>
       </c>
       <c r="F27">
-        <v>0.1489887640583906</v>
+        <v>0.137325901503185</v>
       </c>
       <c r="G27">
-        <v>0.1489887911448457</v>
+        <v>0.1373262344200334</v>
       </c>
       <c r="H27">
-        <v>0.1532017411939513</v>
+        <v>0.1427025486269706</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1215,19 +1215,19 @@
         <v>0</v>
       </c>
       <c r="D29">
-        <v>3.655645070954894E-08</v>
+        <v>5.409397619470515E-08</v>
       </c>
       <c r="E29">
-        <v>2.375382125192369E-07</v>
+        <v>1.298813394802733E-06</v>
       </c>
       <c r="F29">
-        <v>0.0319840633929998</v>
+        <v>0.0362378378655295</v>
       </c>
       <c r="G29">
-        <v>0.0502252984377201</v>
+        <v>0.0502252994975082</v>
       </c>
       <c r="H29">
-        <v>0.0502253005260369</v>
+        <v>0.0502253005580625</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -1319,19 +1319,19 @@
         <v>0</v>
       </c>
       <c r="D33">
-        <v>0.0290687783295164</v>
+        <v>0.0311416245348788</v>
       </c>
       <c r="E33">
-        <v>0.0290687784893082</v>
+        <v>0.03114162477722</v>
       </c>
       <c r="F33">
-        <v>0.0290687787315847</v>
+        <v>0.0311416253577614</v>
       </c>
       <c r="G33">
-        <v>0.0290687789869533</v>
+        <v>0.0311416257879567</v>
       </c>
       <c r="H33">
-        <v>0.0290687828186036</v>
+        <v>0.0311416329372982</v>
       </c>
     </row>
     <row r="34" spans="1:8">

</xml_diff>